<commit_message>
Regenerate all sales docs with new pricing ($299/$599/$1199)
- docs/generate-cashflow.php: updated plan prices (299, 599, 1199)
  and op costs. 'Profesional' rebranded to 'Pro' in tabs.
- docs/generate-vendedor-acuerdo.php: commission multiplier 3× → 1.5×
  (matches Commission::halfAmount in app), updated all plans to
  Free/Básico/Pro/Clínica with new prices. Calculator formula fixed
  to exclude both Free and Básico from commissions.
- NEW: docs/generate-vendedor-kit.php — Complete sales kit Excel
  with 10 sheets: portada, planes, features por plan, features IA,
  vs competencia, script de venta, calculadora ROI, comisiones,
  links y recursos, checklist de venta.

Regenerated files:
- docs/sales-cashflow.xlsx
- docs/acuerdo-vendedor.xlsx
- docs/DocFacil-Kit-Vendedor-2026.xlsx

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/acuerdo-vendedor.xlsx
+++ b/docs/acuerdo-vendedor.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="90">
   <si>
     <t>ACUERDO COMERCIAL — VENDEDOR DocFácil</t>
   </si>
@@ -26,13 +26,13 @@
     <t>1. Esquema de comisión</t>
   </si>
   <si>
-    <t xml:space="preserve">  • La comisión por cada nueva clínica vendida es de 3× la primera mensualidad del plan contratado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • Ejemplo: plan Profesional $299/mes → comisión total $897 por venta.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • Solo aplican los planes Profesional, Clínica y Enterprise. El plan Básico NO paga comisión.</t>
+    <t xml:space="preserve">  • La comisión por cada nueva clínica vendida es de 1.5× la primera mensualidad del plan contratado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Ejemplo: plan Pro $599/mes → comisión total $898.50 por venta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Solo aplican los planes Pro y Clínica. Los planes Free y Básico NO pagan comisión.</t>
   </si>
   <si>
     <t>2. Pago en dos exhibiciones (split 50/50)</t>
@@ -44,7 +44,7 @@
     <t xml:space="preserve">  • 50% (segunda mitad) se paga cuando la clínica realiza su SEGUNDO pago mensual.</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Ejemplo Profesional: $448.50 al 1er pago + $448.50 al 2do pago = $897 total.</t>
+    <t xml:space="preserve">  • Ejemplo Pro: $449.25 al 1er pago + $449.25 al 2do pago = $898.50 total.</t>
   </si>
   <si>
     <t xml:space="preserve">  • Si la clínica NO hace el 2do pago, la segunda mitad no se paga.</t>
@@ -140,7 +140,7 @@
     <t>Precio mensual</t>
   </si>
   <si>
-    <t>Comisión total por venta (3×)</t>
+    <t>Comisión total por venta (1.5×)</t>
   </si>
   <si>
     <t>Primera mitad (50%)</t>
@@ -185,22 +185,22 @@
     <t>EJEMPLOS CONCRETOS</t>
   </si>
   <si>
-    <t xml:space="preserve">  ✓  Si vendes 1 Profesional al mes → 12 × $897 = $10,764/año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ✓  Si vendes 5 Profesional al mes → 60 × $897 = $53,820/año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ✓  Si vendes 10 Profesional al mes → 120 × $897 = $107,640/año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ✓  Si vendes 3 Profesional + 1 Clínica al mes → (3×$897 + 1×$1,497) × 12 = $50,256/año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ✓  Si vendes 5 Clínica al mes → 60 × $1,497 = $89,820/año 🚀</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ✓  Nota: el plan Básico ($149) NO paga comisión — margen insuficiente.</t>
+    <t xml:space="preserve">  ✓  Si vendes 1 Pro al mes → 12 × $898.50 = $10,782/año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ✓  Si vendes 5 Pro al mes → 60 × $898.50 = $53,910/año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ✓  Si vendes 10 Pro al mes → 120 × $898.50 = $107,820/año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ✓  Si vendes 3 Pro + 1 Clínica al mes → (3×$898.50 + 1×$1,798.50) × 12 = $54,126/año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ✓  Si vendes 5 Clínica al mes → 60 × $1,798.50 = $107,910/año 🚀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ✓  Nota: los planes Free ($0) y Básico ($299) NO pagan comisión — margen insuficiente.</t>
   </si>
   <si>
     <t>TRACKING DE VENTAS Y COMISIONES — Captura tus ventas aquí</t>
@@ -257,7 +257,7 @@
     <t>TABLA DE PLANES — Usada por las fórmulas</t>
   </si>
   <si>
-    <t>Comisión total (3×)</t>
+    <t>Comisión total (1.5×)</t>
   </si>
   <si>
     <t>Por mitad (50%)</t>
@@ -266,10 +266,16 @@
     <t>¿Califica?</t>
   </si>
   <si>
+    <t>Free</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
     <t>Básico</t>
   </si>
   <si>
-    <t>NO</t>
+    <t>Pro</t>
   </si>
   <si>
     <t>SÍ</t>
@@ -281,7 +287,7 @@
     <t>NOTA: Solo los planes Profesional, Clínica y Enterprise pagan comisión.</t>
   </si>
   <si>
-    <t>La comisión es 3× la mensualidad, dividida en 2 pagos (al 1er y al 2do pago del cliente).</t>
+    <t>La comisión es 1.5× la mensualidad, dividida en 2 pagos (al 1er y al 2do pago del cliente).</t>
   </si>
 </sst>
 </file>
@@ -1072,8 +1078,8 @@
         <v>39</v>
       </c>
       <c r="E4" s="12">
-        <f>IFERROR(VLOOKUP(B4,Planes!A4:B6,2,FALSE),0)</f>
-        <v>299</v>
+        <f>IFERROR(VLOOKUP(B4,Planes!A4:B7,2,FALSE),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1087,8 +1093,8 @@
         <v>40</v>
       </c>
       <c r="E5" s="13">
-        <f>IF(OR(B4="Básico"),0,E4*3)</f>
-        <v>897</v>
+        <f>IF(OR(B4="Free",B4="Básico"),0,E4*1.5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1103,7 +1109,7 @@
       </c>
       <c r="E6" s="12">
         <f>E5/2</f>
-        <v>448.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1112,7 +1118,7 @@
       </c>
       <c r="E7" s="12">
         <f>E5/2</f>
-        <v>448.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5" customHeight="1" ht="25">
@@ -1147,15 +1153,15 @@
       </c>
       <c r="C11" s="16">
         <f>B11*$E$5</f>
-        <v>8970</v>
+        <v>0</v>
       </c>
       <c r="D11" s="17">
         <f>C11*$B$6</f>
-        <v>8073</v>
+        <v>0</v>
       </c>
       <c r="E11" s="16">
         <f>D11</f>
-        <v>8073</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1168,15 +1174,15 @@
       </c>
       <c r="C12" s="16">
         <f>B12*$E$5</f>
-        <v>26910</v>
+        <v>0</v>
       </c>
       <c r="D12" s="17">
         <f>C12*$B$6</f>
-        <v>24219</v>
+        <v>0</v>
       </c>
       <c r="E12" s="16">
         <f>D12</f>
-        <v>24219</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1189,15 +1195,15 @@
       </c>
       <c r="C13" s="16">
         <f>B13*$E$5</f>
-        <v>53820</v>
+        <v>0</v>
       </c>
       <c r="D13" s="17">
         <f>C13*$B$6</f>
-        <v>48438</v>
+        <v>0</v>
       </c>
       <c r="E13" s="16">
         <f>D13</f>
-        <v>48438</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1210,15 +1216,15 @@
       </c>
       <c r="C14" s="16">
         <f>B14*$E$5</f>
-        <v>107640</v>
+        <v>0</v>
       </c>
       <c r="D14" s="17">
         <f>C14*$B$6</f>
-        <v>96876</v>
+        <v>0</v>
       </c>
       <c r="E14" s="16">
         <f>D14</f>
-        <v>96876</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1231,15 +1237,15 @@
       </c>
       <c r="C15" s="16">
         <f>B15*$E$5</f>
-        <v>215280</v>
+        <v>0</v>
       </c>
       <c r="D15" s="17">
         <f>C15*$B$6</f>
-        <v>193752</v>
+        <v>0</v>
       </c>
       <c r="E15" s="16">
         <f>D15</f>
-        <v>193752</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1292,7 +1298,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" errorStyle="information" operator="between" allowBlank="0" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="B4">
-      <formula1>"Básico,Profesional,Clínica"</formula1>
+      <formula1>"Básico,Pro,Clínica"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
@@ -2251,7 +2257,7 @@
         <v>82</v>
       </c>
       <c r="B4" s="16">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="C4" s="16">
         <v>0</v>
@@ -2265,19 +2271,19 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="15" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="B5" s="16">
         <v>299</v>
       </c>
       <c r="C5" s="16">
-        <v>897</v>
+        <v>0</v>
       </c>
       <c r="D5" s="16">
-        <v>448.5</v>
+        <v>0</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2285,26 +2291,43 @@
         <v>85</v>
       </c>
       <c r="B6" s="16">
-        <v>499</v>
+        <v>599</v>
       </c>
       <c r="C6" s="16">
-        <v>1497</v>
+        <v>898.5</v>
       </c>
       <c r="D6" s="16">
-        <v>748.5</v>
+        <v>449.25</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7">
+        <v>1199</v>
+      </c>
+      <c r="C7">
+        <v>1798.5</v>
+      </c>
+      <c r="D7">
+        <v>899.25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>